<commit_message>
[UEAT] Modify the database_data.xlsx
</commit_message>
<xml_diff>
--- a/user_exp_auto_test_ui/database_data.xlsx
+++ b/user_exp_auto_test_ui/database_data.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="202">
   <si>
     <t>Name</t>
   </si>
@@ -616,6 +616,12 @@
   </si>
   <si>
     <t>x</t>
+  </si>
+  <si>
+    <t>Platform short name</t>
+  </si>
+  <si>
+    <t>short_platform</t>
   </si>
 </sst>
 </file>
@@ -2651,7 +2657,23 @@
         <v>199</v>
       </c>
     </row>
-    <row r="75" ht="14.25" customHeight="1"/>
+    <row r="75" ht="14.25" customHeight="1">
+      <c r="A75" s="41">
+        <v>74.0</v>
+      </c>
+      <c r="B75" s="43" t="s">
+        <v>200</v>
+      </c>
+      <c r="C75" s="43" t="s">
+        <v>201</v>
+      </c>
+      <c r="D75" s="42"/>
+      <c r="E75" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F75" s="42"/>
+      <c r="G75" s="42"/>
+    </row>
     <row r="76" ht="14.25" customHeight="1"/>
     <row r="77" ht="14.25" customHeight="1"/>
     <row r="78" ht="14.25" customHeight="1"/>

</xml_diff>